<commit_message>
Rename the Earth Engine green space indicator from LPUGS to PUGS
- rename the indicator, acronym, database tables and columns, geopackage
  layer, output names and report labels from 'Large Public Urban Green
  Space' (LPUGS) to 'Public Urban Green Space' (PUGS), reflecting that it
  now includes public green space of any size rather than only areas of at
  least one hectare
- the rename covers the sampling functions, the public_urban_green_space
  and pugs_* tables, the *_public_green_space_score output columns, the
  ee_public_green_space_map figure, the download raster and its cache
  directory, the report/data dictionary/workbook labels, and the
  documentation
- also carry the health services accessibility label fix in the same
  files: the PDF page was rendering its label without the city-level
  percentage, so the label phrase now holds the value like the other
  accessibility figures
</commit_message>
<xml_diff>
--- a/process/configuration/assets/output_data_dictionary.xlsx
+++ b/process/configuration/assets/output_data_dictionary.xlsx
@@ -484,7 +484,6 @@
           <t>Continent</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>category</t>
@@ -512,7 +511,6 @@
           <t>Country</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>category</t>
@@ -540,7 +538,6 @@
           <t>ISO 3166-1 alpha-2</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>category</t>
@@ -568,7 +565,6 @@
           <t>study_region</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>category</t>
@@ -948,7 +944,6 @@
           <t>grid_id</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>category</t>
@@ -976,7 +971,6 @@
           <t>point_id</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>category</t>
@@ -1036,9 +1030,6 @@
           <t>[destination]</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1056,8 +1047,6 @@
           <t>fresh_food_market</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>Food (strict)</t>
@@ -1080,8 +1069,6 @@
           <t>fresh_food_pooled</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>Food (lenient)</t>
@@ -1104,8 +1091,6 @@
           <t>convenience</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>Food</t>
@@ -1128,8 +1113,6 @@
           <t>public_open_space_large</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>Open space (strict)</t>
@@ -1152,8 +1135,6 @@
           <t>public_open_space_any</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>Open space (lenient)</t>
@@ -1168,16 +1149,14 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Large public green space (≥ 1 ha; OpenStreetMap and Earth Engine)</t>
+          <t>Public green space (OpenStreetMap and Earth Engine)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>large_public_green_space</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+          <t>public_green_space</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Open space</t>
@@ -1200,8 +1179,6 @@
           <t>pt_frequent</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>Transport (strict, cycling)</t>
@@ -1224,8 +1201,6 @@
           <t>pt_gtfs_freq_20</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Transport (walking)</t>
@@ -1248,8 +1223,6 @@
           <t>pt_gtfs_freq_30</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Transport (walking)</t>
@@ -1272,8 +1245,6 @@
           <t>pt_gtfs_any</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>Transport</t>
@@ -1296,8 +1267,6 @@
           <t>pt_osm_any</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>Transport</t>
@@ -1320,8 +1289,6 @@
           <t>pt_any</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>Transport (lenient)</t>
@@ -1344,8 +1311,6 @@
           <t>all_strict</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>Combined</t>
@@ -1368,8 +1333,6 @@
           <t>all_lenient</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>Combined</t>
@@ -1392,8 +1355,6 @@
           <t>activity_centre_local</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>Derived</t>
@@ -1416,8 +1377,6 @@
           <t>activity_centre_complete</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>Derived</t>
@@ -1435,10 +1394,6 @@
           <t>Regions can define their own destinations (custom OpenStreetMap tags or supplied datasets), pool categories, and configure additional combined-access sets and activity-centre definitions (a network location whose walkable catchment, default 400 m, contains at least one destination of every required category).  These follow the same naming patterns, e.g. all_&lt;set&gt;_&lt;variant&gt; for a named combined-access set and activity_centre_&lt;definition&gt;_&lt;tier&gt; for a named activity centre.  Combined-access composites have access indicators only (no nearest-distance variables).</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1456,9 +1411,6 @@
           <t>[x]</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1476,9 +1428,6 @@
           <t>[network]</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">

</xml_diff>

<commit_message>
Refresh reference data dictionary assets
Regenerate the reference catalogue for the age-friendly access indicators and the updated GUHVI heat exposure description.
</commit_message>
<xml_diff>
--- a/process/configuration/assets/output_data_dictionary.xlsx
+++ b/process/configuration/assets/output_data_dictionary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:F87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -484,6 +484,7 @@
           <t>Continent</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>category</t>
@@ -511,6 +512,7 @@
           <t>Country</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>category</t>
@@ -538,6 +540,7 @@
           <t>ISO 3166-1 alpha-2</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>category</t>
@@ -565,6 +568,7 @@
           <t>study_region</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>category</t>
@@ -944,6 +948,7 @@
           <t>grid_id</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>category</t>
@@ -971,6 +976,7 @@
           <t>point_id</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>category</t>
@@ -1017,17 +1023,32 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Naming conventions and parameters</t>
+          <t>Analytical statistics</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>The destination whose access is measured.  The default destinations are listed below.  Walking and cycling access draw on the same destination definitions, declared once in a region's "accessibility" configuration; each pairs a strict and a lenient variant of each core category (food, public open space, public transport) so that composite "all categories reachable" indicators can be derived per variant.</t>
+          <t>Count of areas of the aggregation summarised here that are associated with this area</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>[destination]</t>
+          <t>area_count</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>custom areas</t>
         </is>
       </c>
     </row>
@@ -1039,19 +1060,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Fresh food market / supermarket</t>
+          <t>The destination whose access is measured.  The default destinations are listed below.  Walking and cycling access draw on the same destination definitions, declared once in a region's "accessibility" configuration; each pairs a strict and a lenient variant of each core category (food, public open space, public transport) so that composite "all categories reachable" indicators can be derived per variant.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>fresh_food_market</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Food (strict)</t>
-        </is>
-      </c>
+          <t>[destination]</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1061,17 +1080,19 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Fresh food, pooled (market, supermarket or convenience store)</t>
+          <t>Fresh food market / supermarket</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>fresh_food_pooled</t>
-        </is>
-      </c>
+          <t>fresh_food_market</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Food (lenient)</t>
+          <t>Food (strict)</t>
         </is>
       </c>
     </row>
@@ -1083,17 +1104,19 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Convenience store</t>
+          <t>Fresh food, pooled (market, supermarket or convenience store)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>convenience</t>
-        </is>
-      </c>
+          <t>fresh_food_pooled</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Food</t>
+          <t>Food (lenient)</t>
         </is>
       </c>
     </row>
@@ -1105,17 +1128,19 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Large public open space (≥ 1.5 ha)</t>
+          <t>Convenience store</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>public_open_space_large</t>
-        </is>
-      </c>
+          <t>convenience</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Open space (strict)</t>
+          <t>Food</t>
         </is>
       </c>
     </row>
@@ -1127,17 +1152,19 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Any public open space</t>
+          <t>Large public open space (≥ 1.5 ha)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>public_open_space_any</t>
-        </is>
-      </c>
+          <t>public_open_space_large</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Open space (lenient)</t>
+          <t>Open space (strict)</t>
         </is>
       </c>
     </row>
@@ -1149,17 +1176,19 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Public green space (OpenStreetMap and Earth Engine)</t>
+          <t>Any public open space</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>public_green_space</t>
-        </is>
-      </c>
+          <t>public_open_space_any</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Open space</t>
+          <t>Open space (lenient)</t>
         </is>
       </c>
     </row>
@@ -1171,17 +1200,19 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Frequent public transport (≤ 20 min daytime service; GTFS)</t>
+          <t>Public green space (OpenStreetMap and Earth Engine)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>pt_frequent</t>
-        </is>
-      </c>
+          <t>public_green_space</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Transport (strict, cycling)</t>
+          <t>Open space</t>
         </is>
       </c>
     </row>
@@ -1193,17 +1224,19 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Public transport, ≤ 20 min daytime service (GTFS)</t>
+          <t>Frequent public transport (≤ 20 min daytime service; GTFS)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>pt_gtfs_freq_20</t>
-        </is>
-      </c>
+          <t>pt_frequent</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Transport (walking)</t>
+          <t>Transport (strict, cycling)</t>
         </is>
       </c>
     </row>
@@ -1215,14 +1248,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Public transport, ≤ 30 min daytime service (GTFS)</t>
+          <t>Public transport, ≤ 20 min daytime service (GTFS)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>pt_gtfs_freq_30</t>
-        </is>
-      </c>
+          <t>pt_gtfs_freq_20</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Transport (walking)</t>
@@ -1237,17 +1272,19 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Any public transport stop (GTFS)</t>
+          <t>Public transport, ≤ 30 min daytime service (GTFS)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>pt_gtfs_any</t>
-        </is>
-      </c>
+          <t>pt_gtfs_freq_30</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Transport</t>
+          <t>Transport (walking)</t>
         </is>
       </c>
     </row>
@@ -1259,14 +1296,16 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Any public transport stop (OpenStreetMap or custom)</t>
+          <t>Any public transport stop (GTFS)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>pt_osm_any</t>
-        </is>
-      </c>
+          <t>pt_gtfs_any</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>Transport</t>
@@ -1281,17 +1320,19 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Any public transport stop (best of GTFS and OpenStreetMap/custom)</t>
+          <t>Any public transport stop (OpenStreetMap or custom)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>pt_any</t>
-        </is>
-      </c>
+          <t>pt_osm_any</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Transport (lenient)</t>
+          <t>Transport</t>
         </is>
       </c>
     </row>
@@ -1303,17 +1344,19 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>All categories reachable, strict variants</t>
+          <t>Any public transport stop (best of GTFS and OpenStreetMap/custom)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>all_strict</t>
-        </is>
-      </c>
+          <t>pt_any</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Combined</t>
+          <t>Transport (lenient)</t>
         </is>
       </c>
     </row>
@@ -1325,14 +1368,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>All categories reachable, lenient variants</t>
+          <t>All categories reachable, strict variants</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>all_lenient</t>
-        </is>
-      </c>
+          <t>all_strict</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>Combined</t>
@@ -1347,17 +1392,19 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Local activity centre (everyday destinations co-located)</t>
+          <t>All categories reachable, lenient variants</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>activity_centre_local</t>
-        </is>
-      </c>
+          <t>all_lenient</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Combined</t>
         </is>
       </c>
     </row>
@@ -1369,14 +1416,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Complete activity centre (high-amenity destinations co-located)</t>
+          <t>Local activity centre (everyday destinations co-located)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>activity_centre_complete</t>
-        </is>
-      </c>
+          <t>activity_centre_local</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>Derived</t>
@@ -1391,7 +1440,19 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Regions can define their own destinations (custom OpenStreetMap tags or supplied datasets), pool categories, and configure additional combined-access sets and activity-centre definitions (a network location whose walkable catchment, default 400 m, contains at least one destination of every required category).  These follow the same naming patterns, e.g. all_&lt;set&gt;_&lt;variant&gt; for a named combined-access set and activity_centre_&lt;definition&gt;_&lt;tier&gt; for a named activity centre.  Combined-access composites have access indicators only (no nearest-distance variables).</t>
+          <t>Complete activity centre (high-amenity destinations co-located)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>activity_centre_complete</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Derived</t>
         </is>
       </c>
     </row>
@@ -1403,14 +1464,13 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Distance threshold (m).  Distances can be customised to locally policy-relevant values.  The core walking access indicators use the configured neighbourhood accessibility threshold (default 500 m).  Where a region configures the optional pedestrian accessibility analysis, walking access is additionally evaluated at each configured pedestrian distance, and cycling access at each configured cycling distance (defaults: 500 m, 1000 m, 2000 m and 5000 m), so an access variable exists for each distance.</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>[x]</t>
-        </is>
-      </c>
+          <t>Regions can define their own destinations (custom OpenStreetMap tags or supplied datasets), pool categories, and configure additional combined-access sets and activity-centre definitions (a network location whose walkable catchment, default 400 m, contains at least one destination of every required category).  These follow the same naming patterns, e.g. all_&lt;set&gt;_&lt;variant&gt; for a named combined-access set and activity_centre_&lt;definition&gt;_&lt;tier&gt; for a named activity centre.  Combined-access composites have access indicators only (no nearest-distance variables).</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1420,46 +1480,37 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Cycling route stress measure, appearing as an optional prefix on cycling variable names: "lts1_" for routes composed entirely of lowest-stress Level of Traffic Stress (LTS) 1 links (suitable for all ages and abilities); "safe_" for fully low-stress routes on LTS 1–2 links (the default headline measure); or no prefix for danger-weighted routing over the full cycling network (higher-stress links usable at a proportionate distance penalty).  Which measures are computed is configurable (cycling_indicators contrasts and measures settings).</t>
+          <t>Distance threshold (m).  Distances can be customised to locally policy-relevant values.  The core walking access indicators use the configured neighbourhood accessibility threshold (default 400 m).  Where a region configures the optional pedestrian accessibility analysis, walking access is additionally evaluated at each configured pedestrian distance, and cycling access at each configured cycling distance (defaults: 400 m, 1000 m, 2000 m and 5000 m), so an access variable exists for each distance.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>[network]</t>
-        </is>
-      </c>
+          <t>[x]</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Indicator estimates: access (walking)</t>
+          <t>Naming conventions and parameters</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Score (0-1) for walking access within the configured accessibility threshold distance (default 500 m) to the destination</t>
+          <t>Cycling route stress measure, appearing as an optional prefix on cycling variable names: "lts1_" for routes composed entirely of lowest-stress Level of Traffic Stress (LTS) 1 links (suitable for all ages and abilities); "safe_" for fully low-stress routes on LTS 1–2 links (the default headline measure); or no prefix for danger-weighted routing over the full cycling network (higher-stress links usable at a proportionate distance penalty).  Which measures are computed is configurable (cycling_indicators contrasts and measures settings).</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>sp_access_[destination]_score</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>score 0-1</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>sample point</t>
-        </is>
-      </c>
+          <t>[network]</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1469,17 +1520,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Distance (m) along the pedestrian network to the nearest destination</t>
+          <t>Score (0-1) for walking access within the configured accessibility threshold distance (default 400 m) to the destination</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>sp_nearest_node_[destination]</t>
+          <t>sp_access_[destination]_score</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>metres</t>
+          <t>score 0-1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1501,27 +1552,27 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Percentage of population with walking access within [x] m of the destination</t>
+          <t>Distance (m) along the pedestrian network to the nearest destination</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>pct_access_[x]m_[destination]_score</t>
+          <t>sp_nearest_node_[destination]</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>metres</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>percentage</t>
+          <t>value</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>grid, custom areas</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
@@ -1533,12 +1584,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Percentage of population with walking access within [x] m of the destination (population weighted)</t>
+          <t>Percentage of population with walking access within [x] m of the destination</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>pop_pct_access_[x]m_[destination]_score</t>
+          <t>pct_access_[x]m_[destination]_score</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1553,7 +1604,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>city, custom areas</t>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
@@ -1565,27 +1616,27 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Score (0/1): the destination is reachable within [x] m along the pedestrian network</t>
+          <t>Percentage of population with walking access within [x] m of the destination (population weighted)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>sp_walk_access_[destination]_[x]m</t>
+          <t>pop_pct_access_[x]m_[destination]_score</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>score 0-1</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>percentage</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>sample point</t>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
@@ -1597,17 +1648,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Distance (m) along the pedestrian network to the nearest destination</t>
+          <t>Score (0/1): the destination is reachable within [x] m along the pedestrian network</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>sp_walk_nearest_node_[destination]</t>
+          <t>sp_walk_access_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>metres</t>
+          <t>score 0-1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1629,27 +1680,27 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Percentage of population with walking access within [x] m to the destination</t>
+          <t>Distance (m) along the pedestrian network to the nearest destination</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>pct_access_walk_[destination]_[x]m</t>
+          <t>sp_walk_nearest_node_[destination]</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>metres</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>percentage</t>
+          <t>value</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>grid, custom areas</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
@@ -1661,12 +1712,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Percentage of population with walking access within [x] m to the destination (population weighted)</t>
+          <t>Percentage of population with walking access within [x] m to the destination</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>pop_pct_access_walk_[destination]_[x]m</t>
+          <t>pct_access_walk_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1681,7 +1732,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>city, custom areas</t>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
@@ -1693,27 +1744,27 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Average distance (m) along the pedestrian network to the nearest destination</t>
+          <t>Percentage of population with walking access within [x] m to the destination (population weighted)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>avg_walk_dist_[destination]</t>
+          <t>pop_pct_access_walk_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>metres</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>percentage</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>grid, custom areas</t>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
@@ -1725,12 +1776,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Average distance (m) along the pedestrian network to the nearest destination (population weighted)</t>
+          <t>Average distance (m) along the pedestrian network to the nearest destination</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>pop_avg_walk_dist_[destination]</t>
+          <t>avg_walk_dist_[destination]</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1745,7 +1796,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>city, custom areas</t>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
@@ -1757,27 +1808,27 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Score (0/1): the nearest destination is further than [x] m along the pedestrian network</t>
+          <t>Average distance (m) along the pedestrian network to the nearest destination (population weighted)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>sp_walk_beyond_[destination]_[x]m</t>
+          <t>pop_avg_walk_dist_[destination]</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>score 0-1</t>
+          <t>metres</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>sample point</t>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
@@ -1789,27 +1840,27 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Percentage of population living further than [x] m along the pedestrian network from the nearest destination</t>
+          <t>Score (0/1): the nearest destination is further than [x] m along the pedestrian network</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>pct_beyond_walk_[destination]_[x]m</t>
+          <t>sp_walk_beyond_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>score 0-1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>percentage</t>
+          <t>value</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>grid, custom areas</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
@@ -1821,12 +1872,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Percentage of population living further than [x] m along the pedestrian network from the nearest destination (population weighted)</t>
+          <t>Percentage of population living further than [x] m along the pedestrian network from the nearest destination</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>pop_pct_beyond_walk_[destination]_[x]m</t>
+          <t>pct_beyond_walk_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1841,7 +1892,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>city, custom areas</t>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
@@ -1853,27 +1904,27 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Number of destinations of the sub-type reachable within [x] m along the pedestrian network</t>
+          <t>Percentage of population living further than [x] m along the pedestrian network from the nearest destination (population weighted)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>sp_walk_count_[set]__[sub-type]_[x]m</t>
+          <t>pop_pct_beyond_walk_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>percentage</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>sample point</t>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
@@ -1885,12 +1936,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Average number of destinations of the sub-type reachable within [x] m along the pedestrian network</t>
+          <t>Number of destinations of the sub-type reachable within [x] m along the pedestrian network</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>avg_count_walk_[set]__[sub-type]_[x]m</t>
+          <t>sp_walk_count_[set]__[sub-type]_[x]m</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1900,12 +1951,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>value</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>grid, custom areas</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
@@ -1917,27 +1968,27 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Diversity (0-1) of the sub-types reachable within [x] m along the pedestrian network: the Shannon entropy of the counts of each sub-type, normalised by the number of sub-types defined</t>
+          <t>Average number of destinations of the sub-type reachable within [x] m along the pedestrian network</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>sp_walk_diversity_[set]_[x]m</t>
+          <t>avg_count_walk_[set]__[sub-type]_[x]m</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>index 0-1</t>
+          <t>count</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>sample point</t>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
@@ -1949,12 +2000,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Average diversity (0-1) of the sub-types reachable within [x] m along the pedestrian network</t>
+          <t>Diversity (0-1) of the sub-types reachable within [x] m along the pedestrian network: the Shannon entropy of the counts of each sub-type, normalised by the number of sub-types defined</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>avg_diversity_walk_[set]_[x]m</t>
+          <t>sp_walk_diversity_[set]_[x]m</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1964,12 +2015,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>value</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>grid, custom areas</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
@@ -1981,12 +2032,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Share (0-1) of the set's sub-types with at least one destination reachable within [x] m along the pedestrian network</t>
+          <t>Average diversity (0-1) of the sub-types reachable within [x] m along the pedestrian network</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>sp_walk_richness_[set]_[x]m</t>
+          <t>avg_diversity_walk_[set]_[x]m</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1996,12 +2047,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>sample point</t>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
@@ -2013,12 +2064,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Average share (0-1) of the set's sub-types with at least one destination reachable within [x] m along the pedestrian network</t>
+          <t>Share (0-1) of the set's sub-types with at least one destination reachable within [x] m along the pedestrian network</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>avg_richness_walk_[set]_[x]m</t>
+          <t>sp_walk_richness_[set]_[x]m</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2028,44 +2079,44 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>value</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>grid, custom areas</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (walking)</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Average population density of the local walkable neighbourhood (population per km², based on the population grid cells intersecting the sample point neighbourhood)</t>
+          <t>Average share (0-1) of the set's sub-types with at least one destination reachable within [x] m along the pedestrian network</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>sp_local_nh_avg_pop_density</t>
+          <t>avg_richness_walk_[set]_[x]m</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>persons per km²</t>
+          <t>index 0-1</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>sample point</t>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
@@ -2077,17 +2128,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Average street intersection density of the local walkable neighbourhood (intersections per km²)</t>
+          <t>Average population density of the local walkable neighbourhood (population per km², based on the population grid cells intersecting the sample point neighbourhood)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>sp_local_nh_avg_intersection_density</t>
+          <t>sp_local_nh_avg_pop_density</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>count per km²</t>
+          <t>persons per km²</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2109,17 +2160,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Daily living score (/3): sum of access scores for fresh food, convenience and public transport destinations</t>
+          <t>Average street intersection density of the local walkable neighbourhood (intersections per km²)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>sp_daily_living_score</t>
+          <t>sp_local_nh_avg_intersection_density</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>score 0-3</t>
+          <t>count per km²</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2141,17 +2192,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Walkability index: sum of z-scores of the daily living score, neighbourhood population density and neighbourhood intersection density</t>
+          <t>Daily living score (/3): sum of access scores for fresh food, convenience and public transport destinations</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>sp_walkability_index</t>
+          <t>sp_daily_living_score</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>index (sum of z-scores)</t>
+          <t>score 0-3</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2173,27 +2224,27 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Average walkable neighbourhood population density (population per km²) of sample points in this area</t>
+          <t>Walkability index: sum of z-scores of the daily living score, neighbourhood population density and neighbourhood intersection density</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>local_nh_population_density</t>
+          <t>sp_walkability_index</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>persons per km²</t>
+          <t>index (sum of z-scores)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>value</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>grid, city, custom areas</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
@@ -2205,17 +2256,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Average walkable neighbourhood intersection density (intersections per km²) of sample points in this area</t>
+          <t>Average walkable neighbourhood population density (population per km²) of sample points in this area</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>local_nh_intersection_density</t>
+          <t>local_nh_population_density</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>count per km²</t>
+          <t>persons per km²</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2237,17 +2288,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Average daily living score (/3) of sample points in this area</t>
+          <t>Average walkable neighbourhood intersection density (intersections per km²) of sample points in this area</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>local_daily_living</t>
+          <t>local_nh_intersection_density</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>score 0-3</t>
+          <t>count per km²</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2269,17 +2320,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Average walkability index of sample points in this area</t>
+          <t>Average daily living score (/3) of sample points in this area</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>local_walkability</t>
+          <t>local_daily_living</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>index (sum of z-scores)</t>
+          <t>score 0-3</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2301,17 +2352,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Average walkable neighbourhood population density (population per km²; population weighted)</t>
+          <t>Average walkability index of sample points in this area</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>pop_nh_pop_density</t>
+          <t>local_walkability</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>persons per km²</t>
+          <t>index (sum of z-scores)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2321,7 +2372,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>city, custom areas</t>
+          <t>grid, city, custom areas</t>
         </is>
       </c>
     </row>
@@ -2333,17 +2384,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Average walkable neighbourhood intersection density (intersections per km²; population weighted)</t>
+          <t>Average walkable neighbourhood population density (population per km²; population weighted)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>pop_nh_intersection_density</t>
+          <t>pop_nh_pop_density</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>count per km²</t>
+          <t>persons per km²</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2365,17 +2416,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Average daily living score (/3; population weighted)</t>
+          <t>Average walkable neighbourhood intersection density (intersections per km²; population weighted)</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>pop_daily_living</t>
+          <t>pop_nh_intersection_density</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>score 0-3</t>
+          <t>count per km²</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2397,17 +2448,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Average walkability index (population weighted)</t>
+          <t>Average daily living score (/3; population weighted)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>pop_walkability</t>
+          <t>pop_daily_living</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>index (sum of z-scores)</t>
+          <t>score 0-3</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2424,22 +2475,22 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Heat Exposure Index (HEI): the heat exposure sub-index, derived from land surface temperature</t>
+          <t>Average walkability index (population weighted)</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>urban_heat_exposure_index</t>
+          <t>pop_walkability</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>index 0-100</t>
+          <t>index (sum of z-scores)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2449,7 +2500,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
@@ -2461,17 +2512,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Land surface temperature (°C): the temperature of the Earth’s surface, indicating the lived experience of heat (Landsat 8 surface reflectance, hottest third of the year)</t>
+          <t>Heat Exposure Index (HEI): the heat exposure sub-index, derived from land surface temperature</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>urban_heat_land_surface_temp_c</t>
+          <t>urban_heat_exposure_index</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>degrees Celsius</t>
+          <t>index 0-100</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -2493,17 +2544,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Heat Sensitivity Index (HSI): the equally weighted heat sensitivity sub-index of land surface albedo, NDVI, NDBI, local climate zone, population density and vulnerable population</t>
+          <t>Land surface temperature (°C): the temperature of the Earth’s surface, indicating the lived experience of heat (Landsat 7/8/9 surface reflectance; hottest third of the year composited over the target year and four preceding years)</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>urban_heat_sensitivity_index</t>
+          <t>urban_heat_land_surface_temp_c</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>index 0-100</t>
+          <t>degrees Celsius</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -2525,17 +2576,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Land surface albedo: solar reflectance, where higher reflectance implies less surface heat retention (inverted, so that higher values indicate greater heat vulnerability)</t>
+          <t>Heat Sensitivity Index (HSI): the equally weighted heat sensitivity sub-index of land surface albedo, NDVI, NDBI, local climate zone, population density and vulnerable population</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>urban_heat_land_surface_albedo</t>
+          <t>urban_heat_sensitivity_index</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>proportion 0-1</t>
+          <t>index 0-100</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -2557,17 +2608,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Normalised Difference Vegetation Index (NDVI): a spectral index of vegetation health and greenness (inverted, so that higher values indicate greater heat vulnerability)</t>
+          <t>Land surface albedo: solar reflectance, where higher reflectance implies less surface heat retention (inverted, so that higher values indicate greater heat vulnerability)</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>urban_heat_ndvi</t>
+          <t>urban_heat_land_surface_albedo</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>index -1 to 1</t>
+          <t>proportion 0-1</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -2589,12 +2640,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Normalised Difference Built-up Index (NDBI): a spectral index of impervious surfaces such as concrete and asphalt</t>
+          <t>Normalised Difference Vegetation Index (NDVI): a spectral index of vegetation health and greenness (inverted, so that higher values indicate greater heat vulnerability)</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>urban_heat_ndbi</t>
+          <t>urban_heat_ndvi</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2621,22 +2672,22 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Local Climate Zone: a standardised classification of land cover typologies for urban heat island studies, ordered from least heat retaining (water) to most heat retaining (bare rock or paved)</t>
+          <t>Normalised Difference Built-up Index (NDBI): a spectral index of impervious surfaces such as concrete and asphalt</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>urban_heat_local_climate_zone_ordered</t>
+          <t>urban_heat_ndbi</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>ordered class</t>
+          <t>index -1 to 1</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -2653,22 +2704,22 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Population density (persons per km²), from the GHS-POP global human settlement population grid</t>
+          <t>Local Climate Zone: a standardised classification of land cover typologies for urban heat island studies, ordered from least heat retaining (water) to most heat retaining (bare rock or paved)</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>urban_heat_population_density_per_sqkm</t>
+          <t>urban_heat_local_climate_zone_ordered</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>persons per km²</t>
+          <t>ordered class</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>category</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -2685,22 +2736,22 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Vulnerable population (%): those most at risk from heat on the basis of age, being the combined proportion of the population aged 0–4 and 65+ years</t>
+          <t>Population density (persons per km²), from the GHS-POP global human settlement population grid</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>urban_heat_vulnerable_pop_pct</t>
+          <t>urban_heat_population_density_per_sqkm</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>persons per km²</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>percentage</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -2717,22 +2768,22 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Adaptive Capability Index (ACI): the equally weighted adaptive capability sub-index of child dependency ratio, subnational Human Development Index and infant mortality rate; higher values indicate lower adaptive capability</t>
+          <t>Vulnerable population (%): those most at risk from heat on the basis of age, being the combined proportion of the population aged 0–4 and 65+ years</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>urban_heat_adaptive_capability_index</t>
+          <t>urban_heat_vulnerable_pop_pct</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>index 0-100</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>percentage</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -2749,17 +2800,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Child dependency ratio: children (aged 0–14 years) relative to the working age population (15–64 years), indicating economic reliance</t>
+          <t>Adaptive Capability Index (ACI): the equally weighted adaptive capability sub-index of child dependency ratio, subnational Human Development Index and infant mortality rate; higher values indicate lower adaptive capability</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>urban_heat_child_dependency_ratio</t>
+          <t>urban_heat_adaptive_capability_index</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>ratio</t>
+          <t>index 0-100</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -2781,17 +2832,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Subnational Human Development Index: human well-being assessed through education, health and standard of living</t>
+          <t>Child dependency ratio: children (aged 0–14 years) relative to the working age population (15–64 years), indicating economic reliance</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>urban_heat_subnational_hdi</t>
+          <t>urban_heat_child_dependency_ratio</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>index 0-100</t>
+          <t>ratio</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -2813,17 +2864,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Infant mortality rate: deaths of children under 1 year of age per 1000 live births, a key indicator of population health</t>
+          <t>Subnational Human Development Index: human well-being assessed through education, health and standard of living</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>urban_heat_infant_mortality_rate</t>
+          <t>urban_heat_subnational_hdi</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>deaths per 1,000 live births</t>
+          <t>index 0-100</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -2845,17 +2896,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Global Urban Heat Vulnerability Index (GUHVI): the equally weighted composite of the Heat Exposure, Heat Sensitivity and Adaptive Capability indices, (HEI + HSI + ACI) / 3</t>
+          <t>Infant mortality rate: deaths of children under 1 year of age per 1000 live births, a key indicator of population health</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>urban_heat_guhvi</t>
+          <t>urban_heat_infant_mortality_rate</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>index 0-100</t>
+          <t>deaths per 1,000 live births</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -2877,22 +2928,22 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Global Urban Heat Vulnerability Index (GUHVI) class, from 1 (least vulnerable) to 5 (most vulnerable)</t>
+          <t>Global Urban Heat Vulnerability Index (GUHVI): the equally weighted composite of the Heat Exposure, Heat Sensitivity and Adaptive Capability indices, (HEI + HSI + ACI) / 3</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>urban_heat_guhvi_class</t>
+          <t>urban_heat_guhvi</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>class 1-5</t>
+          <t>index 0-100</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -2909,25 +2960,57 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
+          <t>Global Urban Heat Vulnerability Index (GUHVI) class, from 1 (least vulnerable) to 5 (most vulnerable)</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>urban_heat_guhvi_class</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>class 1-5</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>sample point, grid, city, custom areas</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Indicator estimates: urban heat vulnerability</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
           <t>Percentage of population in Global Urban Heat Vulnerability Index (GUHVI) class 5, the most vulnerable class</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C87" t="inlineStr">
         <is>
           <t>pct_urban_heat_guhvi_class_5_most_vulnerable</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D87" t="inlineStr">
         <is>
           <t>percent</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="E87" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
+      <c r="F87" t="inlineStr">
         <is>
           <t>grid, city, custom areas</t>
         </is>

</xml_diff>